<commit_message>
feat(modelo): compara hibrido e combinacao e escolhe o do app
</commit_message>
<xml_diff>
--- a/reports/metricas.xlsx
+++ b/reports/metricas.xlsx
@@ -7,7 +7,7 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="resumo" sheetId="1" r:id="rId1"/>
+    <sheet name="configuracoes" sheetId="1" r:id="rId1"/>
     <sheet name="limiares" sheetId="2" r:id="rId2"/>
     <sheet name="recall por origem" sheetId="3" r:id="rId3"/>
   </sheets>
@@ -16,27 +16,54 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="17">
-  <si>
-    <t>metrica</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="26">
+  <si>
+    <t>configuracao</t>
+  </si>
+  <si>
+    <t>precisao</t>
+  </si>
+  <si>
+    <t>recall</t>
+  </si>
+  <si>
+    <t>f1</t>
+  </si>
+  <si>
+    <t>alarmes_falsos</t>
+  </si>
+  <si>
+    <t>golpes_de_sms</t>
+  </si>
+  <si>
+    <t>golpes_de_sms_total</t>
+  </si>
+  <si>
+    <t>tipos_reconhecidos</t>
+  </si>
+  <si>
+    <t>tipos</t>
   </si>
   <si>
     <t>baseline</t>
   </si>
   <si>
-    <t>modelo</t>
-  </si>
-  <si>
-    <t>modelo sem LINK</t>
-  </si>
-  <si>
-    <t>precisao</t>
-  </si>
-  <si>
-    <t>recall</t>
-  </si>
-  <si>
-    <t>f1</t>
+    <t>modelo 0,50</t>
+  </si>
+  <si>
+    <t>modelo 0,45</t>
+  </si>
+  <si>
+    <t>modelo sem LINK 0,50</t>
+  </si>
+  <si>
+    <t>hibrido 0,50</t>
+  </si>
+  <si>
+    <t>hibrido 0,45</t>
+  </si>
+  <si>
+    <t>baseline ou modelo 0,45</t>
   </si>
   <si>
     <t>limiar</t>
@@ -398,10 +425,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -414,47 +441,223 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B2">
         <v>0.85</v>
       </c>
       <c r="C2">
+        <v>0.895</v>
+      </c>
+      <c r="D2">
+        <v>0.872</v>
+      </c>
+      <c r="E2">
+        <v>9</v>
+      </c>
+      <c r="F2">
+        <v>14</v>
+      </c>
+      <c r="G2">
+        <v>17</v>
+      </c>
+      <c r="H2">
+        <v>24</v>
+      </c>
+      <c r="I2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
         <v>0.947</v>
-      </c>
-      <c r="D2">
-        <v>0.944</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3">
-        <v>0.895</v>
       </c>
       <c r="C3">
         <v>0.632</v>
       </c>
       <c r="D3">
+        <v>0.758</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3">
+        <v>5</v>
+      </c>
+      <c r="G3">
+        <v>17</v>
+      </c>
+      <c r="H3">
+        <v>12</v>
+      </c>
+      <c r="I3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4">
+        <v>0.8179999999999999</v>
+      </c>
+      <c r="C4">
+        <v>0.789</v>
+      </c>
+      <c r="D4">
+        <v>0.804</v>
+      </c>
+      <c r="E4">
+        <v>10</v>
+      </c>
+      <c r="F4">
+        <v>11</v>
+      </c>
+      <c r="G4">
+        <v>17</v>
+      </c>
+      <c r="H4">
+        <v>19</v>
+      </c>
+      <c r="I4">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5">
+        <v>0.944</v>
+      </c>
+      <c r="C5">
         <v>0.596</v>
       </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4">
-        <v>0.872</v>
-      </c>
-      <c r="C4">
-        <v>0.758</v>
-      </c>
-      <c r="D4">
+      <c r="D5">
         <v>0.731</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>3</v>
+      </c>
+      <c r="G5">
+        <v>17</v>
+      </c>
+      <c r="H5">
+        <v>10</v>
+      </c>
+      <c r="I5">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6">
+        <v>0.854</v>
+      </c>
+      <c r="C6">
+        <v>0.719</v>
+      </c>
+      <c r="D6">
+        <v>0.781</v>
+      </c>
+      <c r="E6">
+        <v>7</v>
+      </c>
+      <c r="F6">
+        <v>11</v>
+      </c>
+      <c r="G6">
+        <v>17</v>
+      </c>
+      <c r="H6">
+        <v>20</v>
+      </c>
+      <c r="I6">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7">
+        <v>0.84</v>
+      </c>
+      <c r="C7">
+        <v>0.737</v>
+      </c>
+      <c r="D7">
+        <v>0.785</v>
+      </c>
+      <c r="E7">
+        <v>8</v>
+      </c>
+      <c r="F7">
+        <v>11</v>
+      </c>
+      <c r="G7">
+        <v>17</v>
+      </c>
+      <c r="H7">
+        <v>21</v>
+      </c>
+      <c r="I7">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8">
+        <v>0.775</v>
+      </c>
+      <c r="C8">
+        <v>0.965</v>
+      </c>
+      <c r="D8">
+        <v>0.859</v>
+      </c>
+      <c r="E8">
+        <v>16</v>
+      </c>
+      <c r="F8">
+        <v>16</v>
+      </c>
+      <c r="G8">
+        <v>17</v>
+      </c>
+      <c r="H8">
+        <v>26</v>
+      </c>
+      <c r="I8">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -469,28 +672,28 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="B1" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="F1" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="G1" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="H1" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -739,21 +942,21 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="C1" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="B2">
         <v>5</v>
@@ -767,7 +970,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="B3">
         <v>31</v>

</xml_diff>

<commit_message>
fix(modelo): corrige o radical de bloqueio no sinal de ameaca
</commit_message>
<xml_diff>
--- a/reports/metricas.xlsx
+++ b/reports/metricas.xlsx
@@ -462,16 +462,16 @@
         <v>9</v>
       </c>
       <c r="B2">
-        <v>0.85</v>
+        <v>0.836</v>
       </c>
       <c r="C2">
         <v>0.895</v>
       </c>
       <c r="D2">
-        <v>0.872</v>
+        <v>0.864</v>
       </c>
       <c r="E2">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F2">
         <v>14</v>
@@ -578,13 +578,13 @@
         <v>13</v>
       </c>
       <c r="B6">
-        <v>0.854</v>
+        <v>0.857</v>
       </c>
       <c r="C6">
-        <v>0.719</v>
+        <v>0.737</v>
       </c>
       <c r="D6">
-        <v>0.781</v>
+        <v>0.792</v>
       </c>
       <c r="E6">
         <v>7</v>
@@ -596,7 +596,7 @@
         <v>17</v>
       </c>
       <c r="H6">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I6">
         <v>26</v>
@@ -607,16 +607,16 @@
         <v>14</v>
       </c>
       <c r="B7">
-        <v>0.84</v>
+        <v>0.824</v>
       </c>
       <c r="C7">
         <v>0.737</v>
       </c>
       <c r="D7">
-        <v>0.785</v>
+        <v>0.778</v>
       </c>
       <c r="E7">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F7">
         <v>11</v>
@@ -636,16 +636,16 @@
         <v>15</v>
       </c>
       <c r="B8">
-        <v>0.775</v>
+        <v>0.764</v>
       </c>
       <c r="C8">
         <v>0.965</v>
       </c>
       <c r="D8">
-        <v>0.859</v>
+        <v>0.853</v>
       </c>
       <c r="E8">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F8">
         <v>16</v>

</xml_diff>